<commit_message>
Lot 4 : verification des fermetures, remplace 2 prospects disqualifies
Verifie les 35 prospects du lot 4 sur Google Maps : aucune fermeture
definitive. 2 prospects etaient neanmoins disqualifies pour d'autres
raisons decouvertes en verifiant : happytime24.de est un portail/annuaire
allemand generique (l'entreprise associee n'est meme pas en France), et
bernard-agri.com est une chaine confirmee a 4 implantations. Remplaces par
Art & Lunettes (Aix-en-Provence) et Garage Olympic (Grenoble), verifies.
</commit_message>
<xml_diff>
--- a/lot_04.xlsx
+++ b/lot_04.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,8 +98,14 @@
       <color rgb="00111827"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00374151"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +130,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -220,6 +231,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1231,12 +1248,12 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>happytime24.de</t>
+          <t>hoerdtoptique.com</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Christiane's Haarstudio</t>
+          <t>Hoerdt Optique</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1273,34 +1290,34 @@
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>bgcolor= | doctype ancien | non responsive | images .gif | document.write | pas de @media | pas de flex/grid | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (6) | non responsive | &lt;br&gt; en masse | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>hoerdtoptique.com</t>
+          <t>megasun-biarritz.fr</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Hoerdt Optique</t>
+          <t>megaSun</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Bayonne</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr"/>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>64</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G9" s="18" t="n">
         <v>8</v>
@@ -1322,46 +1339,46 @@
       </c>
       <c r="K9" s="22" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (6) | non responsive | &lt;br&gt; en masse | pas de @media | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (12) | doctype ancien | non responsive | pas de @media | pas de flex/grid | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>megasun-biarritz.fr</t>
+          <t>ayu-bienetre.fr</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>megaSun</t>
+          <t>AYU bien-être</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Bayonne</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>64</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="n">
-        <v>51</v>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>49</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
@@ -1371,37 +1388,41 @@
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (12) | doctype ancien | non responsive | pas de @media | pas de flex/grid | aucun radius/ombre</t>
+          <t>layout en tableaux (5) | balises &lt;font&gt; (5) | bgcolor= | sans doctype | non responsive</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>ayu-bienetre.fr</t>
+          <t>aulnoy-optic-chelles.fr</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>AYU bien-être</t>
+          <t>Aulnoy Optic</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
-        </is>
-      </c>
-      <c r="D11" s="17" t="inlineStr"/>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Chelles (77500)</t>
+        </is>
+      </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F11" s="23" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
@@ -1420,45 +1441,41 @@
       </c>
       <c r="K11" s="22" t="inlineStr">
         <is>
-          <t>layout en tableaux (5) | balises &lt;font&gt; (5) | bgcolor= | sans doctype | non responsive</t>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>aulnoy-optic-chelles.fr</t>
+          <t>artetlunettes.fr</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Aulnoy Optic</t>
+          <t>Art &amp; Lunettes</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D12" s="24" t="inlineStr">
-        <is>
-          <t>Chelles (77500)</t>
-        </is>
-      </c>
+          <t>Aix-en-Provence</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F12" s="23" t="n">
-        <v>46</v>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>27</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+        <v>6</v>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -1468,12 +1485,12 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>wordpress 4.9.31</t>
         </is>
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (3) | pas de @media | pas de variables CSS</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2179,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="26" t="inlineStr">
         <is>
           <t>Viroflay (78220)</t>
         </is>
@@ -2251,23 +2268,23 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>bernard-agri.com</t>
+          <t>garage-olympic.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Bernard Matériels Agricoles</t>
+          <t>Garage Olympic</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
@@ -2293,7 +2310,7 @@
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (4) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2538,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="26" t="inlineStr">
         <is>
           <t>Montrouge T (92120)</t>
         </is>

</xml_diff>